<commit_message>
#67 R59, R60 Added in Client BOM.
</commit_message>
<xml_diff>
--- a/Design Files/Relay-10A-Switching-Board-v2.0/BOM/Client-BOM-Relay-10A-Switching-Board-v2.0.xlsx
+++ b/Design Files/Relay-10A-Switching-Board-v2.0/BOM/Client-BOM-Relay-10A-Switching-Board-v2.0.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Iftikhar Ahmed\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\muhunthancanagey-servocontrol\Design Files\Relay-10A-Switching-Board-v2.0\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="316">
   <si>
     <t>#</t>
   </si>
@@ -955,6 +955,18 @@
   </si>
   <si>
     <t>Ceramic Tube Fuse 10A D6.35xL31.75mm Disposable fuses ROHS</t>
+  </si>
+  <si>
+    <t>R59, R60</t>
+  </si>
+  <si>
+    <t>RES 560 OHM 1% 1/16W 0402</t>
+  </si>
+  <si>
+    <t>RC0402FR-07560RL</t>
+  </si>
+  <si>
+    <t>560R</t>
   </si>
 </sst>
 </file>
@@ -1182,9 +1194,6 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1196,6 +1205,9 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1484,7 +1496,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K68"/>
+  <dimension ref="A1:K69"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
@@ -1497,6 +1509,8 @@
     <col min="9" max="9" width="6.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="25.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1508,9 +1522,9 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1580,7 +1594,7 @@
     <row r="4" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
-        <f t="shared" ref="B4:B63" si="0">ROW(B4) - ROW($B$2)</f>
+        <f t="shared" ref="B4:B64" si="0">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
       <c r="C4" s="13" t="s">
@@ -3056,28 +3070,28 @@
       <c r="C50" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="D50" s="15" t="s">
+      <c r="D50" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="E50" s="16" t="s">
+      <c r="E50" s="15" t="s">
         <v>131</v>
       </c>
-      <c r="F50" s="15" t="s">
+      <c r="F50" s="14" t="s">
         <v>178</v>
       </c>
-      <c r="G50" s="16" t="s">
+      <c r="G50" s="15" t="s">
         <v>223</v>
       </c>
-      <c r="H50" s="15" t="s">
+      <c r="H50" s="14" t="s">
         <v>240</v>
       </c>
-      <c r="I50" s="16" t="s">
+      <c r="I50" s="15" t="s">
         <v>286</v>
       </c>
-      <c r="J50" s="15">
-        <v>1</v>
-      </c>
-      <c r="K50" s="18" t="s">
+      <c r="J50" s="14">
+        <v>1</v>
+      </c>
+      <c r="K50" s="17" t="s">
         <v>297</v>
       </c>
     </row>
@@ -3212,446 +3226,477 @@
     <row r="55" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="1"/>
       <c r="B55" s="11">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="B55" si="1">ROW(B55) - ROW($B$2)</f>
         <v>53</v>
       </c>
       <c r="C55" s="13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D55" s="9" t="s">
-        <v>76</v>
+        <v>312</v>
       </c>
       <c r="E55" s="10" t="s">
-        <v>138</v>
+        <v>313</v>
       </c>
       <c r="F55" s="9" t="s">
-        <v>295</v>
+        <v>178</v>
       </c>
       <c r="G55" s="10" t="s">
-        <v>182</v>
+        <v>314</v>
       </c>
       <c r="H55" s="9" t="s">
-        <v>259</v>
+        <v>240</v>
       </c>
       <c r="I55" s="10" t="s">
-        <v>296</v>
+        <v>315</v>
       </c>
       <c r="J55" s="9">
         <v>2</v>
       </c>
       <c r="K55" s="9"/>
     </row>
-    <row r="56" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1"/>
       <c r="B56" s="11">
-        <f>ROW(B56) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>54</v>
       </c>
-      <c r="C56" s="12" t="s">
+      <c r="C56" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="D56" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="E56" s="8" t="s">
-        <v>139</v>
+      <c r="D56" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="E56" s="10" t="s">
+        <v>138</v>
       </c>
       <c r="F56" s="9" t="s">
         <v>295</v>
       </c>
-      <c r="G56" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="H56" s="7" t="s">
-        <v>265</v>
+      <c r="G56" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="H56" s="9" t="s">
+        <v>259</v>
       </c>
       <c r="I56" s="10" t="s">
         <v>296</v>
       </c>
-      <c r="J56" s="7">
-        <v>1</v>
-      </c>
-      <c r="K56" s="7"/>
-    </row>
-    <row r="57" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J56" s="9">
+        <v>2</v>
+      </c>
+      <c r="K56" s="9"/>
+    </row>
+    <row r="57" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1"/>
       <c r="B57" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B57) - ROW($B$2)</f>
         <v>55</v>
       </c>
-      <c r="C57" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="D57" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="E57" s="10" t="s">
-        <v>140</v>
+      <c r="C57" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="D57" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="E57" s="8" t="s">
+        <v>139</v>
       </c>
       <c r="F57" s="9" t="s">
-        <v>184</v>
-      </c>
-      <c r="G57" s="10" t="s">
-        <v>230</v>
-      </c>
-      <c r="H57" s="9" t="s">
-        <v>266</v>
+        <v>295</v>
+      </c>
+      <c r="G57" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="H57" s="7" t="s">
+        <v>265</v>
       </c>
       <c r="I57" s="10" t="s">
         <v>296</v>
       </c>
-      <c r="J57" s="9">
-        <v>1</v>
-      </c>
-      <c r="K57" s="9"/>
-    </row>
-    <row r="58" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J57" s="7">
+        <v>1</v>
+      </c>
+      <c r="K57" s="7"/>
+    </row>
+    <row r="58" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="1"/>
       <c r="B58" s="11">
-        <f>ROW(B58) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>56</v>
       </c>
-      <c r="C58" s="12" t="s">
+      <c r="C58" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="D58" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="E58" s="8" t="s">
-        <v>141</v>
-      </c>
-      <c r="F58" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="G58" s="8" t="s">
-        <v>231</v>
-      </c>
-      <c r="H58" s="7" t="s">
-        <v>244</v>
+      <c r="D58" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="E58" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="F58" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="G58" s="10" t="s">
+        <v>230</v>
+      </c>
+      <c r="H58" s="9" t="s">
+        <v>266</v>
       </c>
       <c r="I58" s="10" t="s">
         <v>296</v>
       </c>
-      <c r="J58" s="7">
-        <v>1</v>
-      </c>
-      <c r="K58" s="7"/>
+      <c r="J58" s="9">
+        <v>1</v>
+      </c>
+      <c r="K58" s="9"/>
     </row>
     <row r="59" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="1"/>
       <c r="B59" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B59) - ROW($B$2)</f>
         <v>57</v>
       </c>
-      <c r="C59" s="13" t="s">
+      <c r="C59" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="D59" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="E59" s="10" t="s">
-        <v>142</v>
-      </c>
-      <c r="F59" s="9" t="s">
-        <v>186</v>
-      </c>
-      <c r="G59" s="10" t="s">
-        <v>232</v>
-      </c>
-      <c r="H59" s="9" t="s">
-        <v>250</v>
+      <c r="D59" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E59" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="F59" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="G59" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="H59" s="7" t="s">
+        <v>244</v>
       </c>
       <c r="I59" s="10" t="s">
         <v>296</v>
       </c>
-      <c r="J59" s="9">
-        <v>1</v>
-      </c>
-      <c r="K59" s="9"/>
+      <c r="J59" s="7">
+        <v>1</v>
+      </c>
+      <c r="K59" s="7"/>
     </row>
     <row r="60" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="1"/>
       <c r="B60" s="11">
-        <f>ROW(B60) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>58</v>
       </c>
-      <c r="C60" s="12" t="s">
+      <c r="C60" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="D60" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="E60" s="8" t="s">
-        <v>143</v>
-      </c>
-      <c r="F60" s="7" t="s">
-        <v>187</v>
-      </c>
-      <c r="G60" s="8" t="s">
-        <v>233</v>
-      </c>
-      <c r="H60" s="7" t="s">
-        <v>266</v>
+      <c r="D60" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="E60" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="F60" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="G60" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="H60" s="9" t="s">
+        <v>250</v>
       </c>
       <c r="I60" s="10" t="s">
         <v>296</v>
       </c>
-      <c r="J60" s="7">
-        <v>1</v>
-      </c>
-      <c r="K60" s="7"/>
+      <c r="J60" s="9">
+        <v>1</v>
+      </c>
+      <c r="K60" s="9"/>
     </row>
     <row r="61" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="1"/>
       <c r="B61" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B61) - ROW($B$2)</f>
         <v>59</v>
       </c>
-      <c r="C61" s="13" t="s">
+      <c r="C61" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="D61" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="E61" s="10" t="s">
+      <c r="D61" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="E61" s="8" t="s">
         <v>143</v>
       </c>
-      <c r="F61" s="9" t="s">
+      <c r="F61" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="G61" s="10" t="s">
-        <v>234</v>
-      </c>
-      <c r="H61" s="9" t="s">
+      <c r="G61" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="H61" s="7" t="s">
         <v>266</v>
       </c>
       <c r="I61" s="10" t="s">
         <v>296</v>
       </c>
-      <c r="J61" s="9">
-        <v>1</v>
-      </c>
-      <c r="K61" s="9"/>
+      <c r="J61" s="7">
+        <v>1</v>
+      </c>
+      <c r="K61" s="7"/>
     </row>
     <row r="62" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="1"/>
       <c r="B62" s="11">
-        <f>ROW(B62) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>60</v>
       </c>
-      <c r="C62" s="12" t="s">
+      <c r="C62" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="D62" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="E62" s="8" t="s">
-        <v>144</v>
-      </c>
-      <c r="F62" s="7" t="s">
-        <v>188</v>
-      </c>
-      <c r="G62" s="8" t="s">
-        <v>235</v>
-      </c>
-      <c r="H62" s="7" t="s">
-        <v>250</v>
+      <c r="D62" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="E62" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="F62" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="G62" s="10" t="s">
+        <v>234</v>
+      </c>
+      <c r="H62" s="9" t="s">
+        <v>266</v>
       </c>
       <c r="I62" s="10" t="s">
         <v>296</v>
       </c>
-      <c r="J62" s="7">
-        <v>1</v>
-      </c>
-      <c r="K62" s="7"/>
+      <c r="J62" s="9">
+        <v>1</v>
+      </c>
+      <c r="K62" s="9"/>
     </row>
     <row r="63" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="1"/>
       <c r="B63" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B63) - ROW($B$2)</f>
         <v>61</v>
       </c>
-      <c r="C63" s="13" t="s">
+      <c r="C63" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="D63" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="E63" s="10" t="s">
-        <v>145</v>
-      </c>
-      <c r="F63" s="9" t="s">
-        <v>189</v>
-      </c>
-      <c r="G63" s="10" t="s">
-        <v>236</v>
-      </c>
-      <c r="H63" s="9" t="s">
-        <v>266</v>
+      <c r="D63" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="E63" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="F63" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="G63" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="H63" s="7" t="s">
+        <v>250</v>
       </c>
       <c r="I63" s="10" t="s">
         <v>296</v>
       </c>
-      <c r="J63" s="9">
-        <v>1</v>
-      </c>
-      <c r="K63" s="9"/>
-    </row>
-    <row r="64" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J63" s="7">
+        <v>1</v>
+      </c>
+      <c r="K63" s="7"/>
+    </row>
+    <row r="64" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A64" s="1"/>
       <c r="B64" s="11">
-        <f>ROW(B64) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>62</v>
       </c>
-      <c r="C64" s="12" t="s">
+      <c r="C64" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="D64" s="7" t="s">
+      <c r="D64" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="E64" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="F64" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="G64" s="10" t="s">
+        <v>236</v>
+      </c>
+      <c r="H64" s="9" t="s">
+        <v>266</v>
+      </c>
+      <c r="I64" s="10" t="s">
+        <v>296</v>
+      </c>
+      <c r="J64" s="9">
+        <v>1</v>
+      </c>
+      <c r="K64" s="9"/>
+    </row>
+    <row r="65" spans="2:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B65" s="11">
+        <f>ROW(B65) - ROW($B$2)</f>
+        <v>63</v>
+      </c>
+      <c r="C65" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D65" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="E64" s="8" t="s">
+      <c r="E65" s="8" t="s">
         <v>146</v>
-      </c>
-      <c r="F64" s="9" t="s">
-        <v>295</v>
-      </c>
-      <c r="G64" s="8" t="s">
-        <v>190</v>
-      </c>
-      <c r="H64" s="7" t="s">
-        <v>267</v>
-      </c>
-      <c r="I64" s="10" t="s">
-        <v>296</v>
-      </c>
-      <c r="J64" s="7">
-        <v>1</v>
-      </c>
-      <c r="K64" s="7"/>
-    </row>
-    <row r="65" spans="2:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B65" s="11">
-        <f t="shared" ref="B65" si="1">ROW(B65) - ROW($B$2)</f>
-        <v>63</v>
-      </c>
-      <c r="C65" s="13" t="s">
-        <v>298</v>
-      </c>
-      <c r="D65" s="9" t="s">
-        <v>299</v>
-      </c>
-      <c r="E65" s="10" t="s">
-        <v>309</v>
       </c>
       <c r="F65" s="9" t="s">
         <v>295</v>
       </c>
-      <c r="G65" s="10" t="s">
-        <v>308</v>
-      </c>
-      <c r="H65" s="9" t="s">
-        <v>252</v>
+      <c r="G65" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="H65" s="7" t="s">
+        <v>267</v>
       </c>
       <c r="I65" s="10" t="s">
         <v>296</v>
       </c>
-      <c r="J65" s="9">
-        <v>1</v>
-      </c>
-      <c r="K65" s="9"/>
+      <c r="J65" s="7">
+        <v>1</v>
+      </c>
+      <c r="K65" s="7"/>
     </row>
     <row r="66" spans="2:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B66" s="11">
-        <f>ROW(B66) - ROW($B$2)</f>
+        <f t="shared" ref="B66" si="2">ROW(B66) - ROW($B$2)</f>
         <v>64</v>
       </c>
       <c r="C66" s="13" t="s">
         <v>298</v>
       </c>
-      <c r="D66" s="7" t="s">
-        <v>300</v>
-      </c>
-      <c r="E66" s="8" t="s">
-        <v>301</v>
+      <c r="D66" s="9" t="s">
+        <v>299</v>
+      </c>
+      <c r="E66" s="10" t="s">
+        <v>309</v>
       </c>
       <c r="F66" s="9" t="s">
         <v>295</v>
       </c>
-      <c r="G66" s="8" t="s">
-        <v>302</v>
-      </c>
-      <c r="H66" s="7" t="s">
-        <v>303</v>
+      <c r="G66" s="10" t="s">
+        <v>308</v>
+      </c>
+      <c r="H66" s="9" t="s">
+        <v>252</v>
       </c>
       <c r="I66" s="10" t="s">
         <v>296</v>
       </c>
-      <c r="J66" s="7">
-        <v>2</v>
-      </c>
-      <c r="K66" s="7"/>
-    </row>
-    <row r="67" spans="2:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J66" s="9">
+        <v>1</v>
+      </c>
+      <c r="K66" s="9"/>
+    </row>
+    <row r="67" spans="2:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B67" s="11">
-        <f t="shared" ref="B67" si="2">ROW(B67) - ROW($B$2)</f>
+        <f>ROW(B67) - ROW($B$2)</f>
         <v>65</v>
       </c>
       <c r="C67" s="13" t="s">
         <v>298</v>
       </c>
       <c r="D67" s="7" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E67" s="8" t="s">
-        <v>311</v>
+        <v>301</v>
       </c>
       <c r="F67" s="9" t="s">
         <v>295</v>
       </c>
       <c r="G67" s="8" t="s">
-        <v>310</v>
+        <v>302</v>
       </c>
       <c r="H67" s="7" t="s">
-        <v>252</v>
-      </c>
-      <c r="I67" s="8" t="s">
+        <v>303</v>
+      </c>
+      <c r="I67" s="10" t="s">
         <v>296</v>
       </c>
       <c r="J67" s="7">
-        <v>4</v>
-      </c>
-      <c r="K67" s="17"/>
-    </row>
-    <row r="68" spans="2:11" ht="64.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+      <c r="K67" s="7"/>
+    </row>
+    <row r="68" spans="2:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B68" s="11">
-        <f>ROW(B68) - ROW($B$2)</f>
+        <f t="shared" ref="B68" si="3">ROW(B68) - ROW($B$2)</f>
         <v>66</v>
       </c>
       <c r="C68" s="13" t="s">
         <v>298</v>
       </c>
       <c r="D68" s="7" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="E68" s="8" t="s">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="F68" s="9" t="s">
         <v>295</v>
       </c>
       <c r="G68" s="8" t="s">
+        <v>310</v>
+      </c>
+      <c r="H68" s="7" t="s">
+        <v>252</v>
+      </c>
+      <c r="I68" s="8" t="s">
+        <v>296</v>
+      </c>
+      <c r="J68" s="7">
+        <v>4</v>
+      </c>
+      <c r="K68" s="16"/>
+    </row>
+    <row r="69" spans="2:11" ht="64.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B69" s="11">
+        <f>ROW(B69) - ROW($B$2)</f>
+        <v>67</v>
+      </c>
+      <c r="C69" s="13" t="s">
+        <v>298</v>
+      </c>
+      <c r="D69" s="7" t="s">
+        <v>304</v>
+      </c>
+      <c r="E69" s="8" t="s">
+        <v>305</v>
+      </c>
+      <c r="F69" s="9" t="s">
+        <v>295</v>
+      </c>
+      <c r="G69" s="8" t="s">
         <v>306</v>
       </c>
-      <c r="H68" s="7" t="s">
-        <v>296</v>
-      </c>
-      <c r="I68" s="8" t="s">
-        <v>296</v>
-      </c>
-      <c r="J68" s="7">
-        <v>1</v>
-      </c>
-      <c r="K68" s="17" t="s">
+      <c r="H69" s="7" t="s">
+        <v>296</v>
+      </c>
+      <c r="I69" s="8" t="s">
+        <v>296</v>
+      </c>
+      <c r="J69" s="7">
+        <v>1</v>
+      </c>
+      <c r="K69" s="16" t="s">
         <v>307</v>
       </c>
     </row>

</xml_diff>